<commit_message>
PLAN_V11 Phase 67: Profilabhängige Anhänge und CS8800-Broschüre
Blatt Anhänge hat die neue Spalte Nicht bei Profil (kommagetrennt):
Broschüre Ratenkauf.pdf und Friondo SpotDynamic.pdf gehen nicht mehr an
Enni und SWD; die Engine filtert beim Zusammenstellen der Mail-Anhänge
(Einzel- und Kombi-Versand sowie Editor-Anzeige) über den Profilnamen
des Angebots. Neue Anhangszeile Bosch CS8800iAW.pdf bei Pos. 030 oder
031 im Angebot; die Datei fehlt noch (Zulieferung 3), bis dahin greift
die bestehende Datei-fehlt-Warnung. VK-Preislisten-Import wartet auf
Zulieferung 2 (Checkbox offen). Phasentest 13/13, Unit-Suite 99/99.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/konfigurator_logik_v5.xlsx
+++ b/konfigurator_logik_v5.xlsx
@@ -8354,7 +8354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -8378,72 +8378,87 @@
           <t>Bemerkung</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Nicht bei Profil</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Friondo Unternehmenspräsentation.pdf</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Unternehmenspräsentation – geht mit jedem Angebot</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Broschüre Ratenkauf.pdf</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Zahlungsoptionen Barkauf/Finanzierung (Nachtext A) – jedes Angebot</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Enni, SWD</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Friondo HEMS.pdf</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>wenn P01 = Ja</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Friondo-HEMS-Broschüre</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Friondo SpotDynamic.pdf</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>wenn P03 = Ja</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>SpotDynamic-Broschüre (dynamischer Stromtarif)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Enni, SWD</t>
         </is>
       </c>
     </row>
@@ -8467,15 +8482,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Bosch CS8800iAW.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>wenn Pos. 030–031 im Angebot</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Gerätebroschüre Serie CS8800i (Datei folgt – Zulieferung 3; bis dahin greift die Datei-fehlt-Warnung)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>(weitere Zeilen ergänzen)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Regeln: 'immer' | 'wenn &lt;Frage&gt; = &lt;Antwort&gt;' | 'wenn Pos. &lt;Nr&gt; im Angebot'</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>PDFs in den Ordner anlagen/ legen</t>
         </is>

</xml_diff>

<commit_message>
PLAN_V13 Phase 79: Prozessintegration PV (Ampel-Weg, Erneut pruefen, Anhaenge)
PV-Katalog-Erfassungen laufen ueber die Ampel (gruen -> Angebot erzeugen, orange -> Individuell);
Button Erneut pruefen fuer Katalog-Erfassungen (PV-Altfaelle bleiben unberuehrt bis zur Pruefung);
Anhangs-/Vollmacht-Regeln greifen ueber PA11-PA13; Anhangsregel wenn Sparte = PV +
Platzhalterzeile Sigenergy-/Modul-Datenblatt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/konfigurator_logik_v5.xlsx
+++ b/konfigurator_logik_v5.xlsx
@@ -15900,7 +15900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -16045,15 +16045,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>(Sigenergy-/Modul-Datenblatt – Zulieferung)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>wenn Sparte = PV</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>v13-PV: Datei nach Lieferung in anlagen/ legen und diese Zeile mit dem Dateinamen füllen (Klammern entfernen) – geht dann mit jedem PV-Angebot mit</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>(weitere Zeilen ergänzen)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Regeln: 'immer' | 'wenn &lt;Frage&gt; = &lt;Antwort&gt;' | 'wenn Pos. &lt;Nr&gt; im Angebot'</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>PDFs in den Ordner anlagen/ legen</t>
         </is>

</xml_diff>

<commit_message>
Rueckfragen 30.09.: Kunden-Dubletten, BzA-Mail-Haekchen, Standard-Sub, AD-Anschriften
- Parametrierung -> Kunden-Dubletten (app/kunden_dubletten.py): Gruppen
  Name + PLZ, Hauptdatensatz waehlbar, Verweise umhaengen, Felder ergaenzen,
  Dubletten loeschen, Protokoll; abweichende Strasse nicht vorausgewaehlt
- BzA-Kundenmail per Haekchen (bza_mail_aktiv), Knopf ohne Mail abschliessen
- Go-live-Checkliste prueft das echte Standard-Kennzeichen je Sub-Typ
- Standard-Anschriften auch fuer den Aussendienst (eigene Vorgaenge)
- BAFA: weisse 8800er ohne eigene Nummer bestaetigt (Hinweis im Blatt)
- tests/test_rueckfragen_0930.py, Doku

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/konfigurator_logik_v5.xlsx
+++ b/konfigurator_logik_v5.xlsx
@@ -727,7 +727,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -768,7 +767,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -809,7 +807,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -850,7 +847,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -891,7 +887,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -932,7 +927,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -973,7 +967,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1014,7 +1007,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1055,7 +1047,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1096,7 +1087,6 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1139,7 +1129,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>PRÜFPUNKT: Zusatz „(B)“ – gilt vorerst für weiße (030) und schwarze (031) Außeneinheit; eigene Nummer der weißen klären</t>
+          <t>gilt für weiße (Pos. 030) und schwarze (Pos. 031) Außeneinheit – keine eigene Nummer (bestätigt 30.09.2026)</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1174,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>PRÜFPUNKT: Zusatz „(B)“ – gilt vorerst für weiße (030) und schwarze (031) Außeneinheit; eigene Nummer der weißen klären</t>
+          <t>gilt für weiße (Pos. 030) und schwarze (Pos. 031) Außeneinheit – keine eigene Nummer (bestätigt 30.09.2026)</t>
         </is>
       </c>
     </row>
@@ -1212,9 +1202,6 @@
       <c r="E14" t="n">
         <v>21</v>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>Vorrat – geplante Klassenerweiterung (Komponenten/Preise offen)</t>
@@ -10974,7 +10961,6 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>immer</t>

</xml_diff>

<commit_message>
v22: Wirtschaftlichkeit PV, PA04, Editor-/BzA-Feedback (PLAN_V15, Phasen 99-103)
Rechenkern mit Saisonmodell (Monatsprofile), drei PDF-Seiten (Poppins), PA04 nur Protokoll, Haekchen + PV-Parameter-Ansicht, Fehlerprotokoll + database-is-locked-Absicherung, Editor-Scroll, Gruppen-Ueberschriften, psl., BzA-Dialog uebersteuerbar, Signatur-Altpfade (Voll-Crawl-Befund).
</commit_message>
<xml_diff>
--- a/konfigurator_logik_v5.xlsx
+++ b/konfigurator_logik_v5.xlsx
@@ -9554,12 +9554,12 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>AMPEL: individuell – Grund: Ertüchtigung bestehender ZV – Positionen noch nicht hinterlegt</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>[OFFEN] Positionen für Ertüchtigung/APZ/HAK-Leitung (PA05/PA06) noch festzulegen</t>
+          <t>v22 (30.09.2026): Ja löst keine Positionen und keine Ampel aus – Antwort nur im Protokoll</t>
         </is>
       </c>
       <c r="E20" s="8" t="n"/>
@@ -10076,7 +10076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -10331,7 +10331,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>[ANNAHME] Unternehmenspräsentation – Basisquote PV</t>
+          <t>[ANNAHME] Unternehmenspräsentation – Basisquote PV – überholt durch Energiebilanz (v22), ungenutzt</t>
         </is>
       </c>
     </row>
@@ -10351,7 +10351,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>[ANNAHME] additiv, wenn ein Speicher im Angebot ist</t>
+          <t>[ANNAHME] additiv, wenn ein Speicher im Angebot ist – überholt durch Energiebilanz (v22), ungenutzt</t>
         </is>
       </c>
     </row>
@@ -10371,7 +10371,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>[ANNAHME] additiv, wenn Friondo HEMS (Pos. 015) im Angebot ist</t>
+          <t>[ANNAHME] additiv, wenn Friondo HEMS (Pos. 015) im Angebot ist – überholt durch Energiebilanz (v22), ungenutzt</t>
         </is>
       </c>
     </row>
@@ -10434,6 +10434,498 @@
       <c r="D18" s="8" t="inlineStr">
         <is>
           <t>aus dem Musterangebot – wird an die Modulposition angehängt</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Strompreissteigerung</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>%/Jahr</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>v22 Wirtschaftlichkeit: Annahme Strompreisentwicklung</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Degradation</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>%/Jahr</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>v22: Leistungsabnahme der Module je Jahr</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Betriebskosten</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>€/Jahr</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>v22: Versicherung, Wartung, Zählergebühr (pauschal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Betrachtungszeitraum</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Jahre</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>v22: Laufzeit der Betrachtung</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Inbetriebnahme-Versatz</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Jahr</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>v22: Startjahr = Angebotsjahr + Versatz</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Direktanteil Haushalt</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>v22: Anteil des Haushaltsstroms, der direkt aus PV gedeckt wird</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Direktanteil Wärmepumpe</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>v22: Anteil des WP-Stroms direkt aus PV (ohne HEMS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Direktanteil Wallbox</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>v22 [ANNAHME]: Anteil des Wallbox-Stroms direkt aus PV</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>HEMS-Zuschlag Haushalt</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>%-Punkte</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>v22: Zuschlag auf den Direktanteil mit Friondo HEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>HEMS-Zuschlag Wärmepumpe</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>%-Punkte</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>v22: Zuschlag auf den Direktanteil mit Friondo HEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>HEMS-Zuschlag Wallbox</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>%-Punkte</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>v22 [ANNAHME]: Zuschlag auf den Direktanteil mit Friondo HEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Speicher Vollzyklen</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>/Jahr</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>v22: nutzbare Vollzyklen des Speichers je Jahr</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Speicher Wirkungsgrad</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>v22: Round-trip-Wirkungsgrad des Speichers</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>SpotDynamic Bezugspreis</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>€/kWh</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>v22: Ø Netzbezugspreis mit Friondo SpotDynamic</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Kosten-Airbag</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>€/kWh</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>v22: Obergrenze SpotDynamic (nur Text auf Seite 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Szenarien Strompreissteigerung</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>1; 3; 5</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>%/Jahr</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>v22: drei Säulen auf Seite 3 (vorsichtig · Ihre Rechnung · stark)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>CO₂-Faktor Netzstrom</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>g/kWh</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>v22: Umweltbundesamt, deutscher Strommix</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>CO₂ Auto</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>g/km</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>v22: Umrechnung in Autokilometer</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>CO₂ Baum</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>kg/Jahr</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>v22: CO₂-Bindung je Baum und Jahr</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Montagedauer-Text</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Montage in 1–2 Tagen</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>v22: Schritt 3 unter „So geht es weiter“ (Seite 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>Monatsprofil PV</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>2,5; 4,5; 10; 11; 12,5; 13; 13; 11,5; 9,5; 7; 3,5; 2</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>% je Monat</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>v22 Saisonmodell: Anteil des Jahresertrags je Monat Jan–Dez (typische Verteilung Deutschland: Nov–Feb ≈ 12 %, Apr–Sep ≈ 70 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Monatsprofil Haushalt</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>9,5; 8,5; 8,8; 8; 7,7; 7,3; 7,5; 7,5; 7,7; 8,4; 9; 10,1</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>% je Monat</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>v22 Saisonmodell [ANNAHME]: Haushaltsstrom je Monat, angelehnt an BDEW-Lastprofil H0 (Winter höher, Sommer niedriger)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>Monatsprofil Wärmepumpe</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>15,3; 13,7; 12,1; 8,1; 4,9; 2,7; 2,7; 2,7; 4,1; 8,1; 11,3; 14,5</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>% je Monat</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>v22 Saisonmodell: 80 % Heizung nach VDI-2067-Gradtagszahlen + 20 % Warmwasser gleichverteilt</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>Monatsprofil Wallbox</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>8,33; 8,33; 8,33; 8,33; 8,33; 8,33; 8,33; 8,33; 8,33; 8,33; 8,33; 8,33</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>% je Monat</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>v22 Saisonmodell [ANNAHME]: Wallbox gleichverteilt</t>
         </is>
       </c>
     </row>

</xml_diff>